<commit_message>
Daily cockpit update 2026-07-22
Edition #10: 31 new stories across all 12 verticals, deduplicated
against the historical log (0 duplicates found). Updates story-log.csv
(now 228 rows), regenerates the rolling last-30-days xlsx export, and
adds today's cockpit-2026-07-22.html.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LhDAjo836xuBHQsr8UERph
</commit_message>
<xml_diff>
--- a/cockpit-data/story-log-last30days.xlsx
+++ b/cockpit-data/story-log-last30days.xlsx
@@ -10,7 +10,9 @@
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Raw Rows (Last 30 Days)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Raw Rows (Last 30 Days)'!$A$1:$I$229</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -58,6 +60,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00004B87"/>
+        <bgColor rgb="00004B87"/>
       </patternFill>
     </fill>
   </fills>
@@ -444,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -461,7 +464,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Window: 2026-06-08 to 2026-07-08</t>
+          <t>Window: 2026-06-22 to 2026-07-22</t>
         </is>
       </c>
     </row>
@@ -491,7 +494,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7">
@@ -501,7 +504,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8">
@@ -511,7 +514,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9">
@@ -521,27 +524,27 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Insurtech</t>
+          <t>Healthcare / Provider &amp; Clinical</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Healthcare / Provider &amp; Clinical</t>
+          <t>Insurtech</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12">
@@ -551,7 +554,7 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13">
@@ -561,37 +564,37 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Investments</t>
+          <t>BrokerTech</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>BrokerTech</t>
+          <t>FinTech</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>FinTech</t>
+          <t>Investments</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17">
@@ -601,7 +604,7 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20">
@@ -630,7 +633,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>41</v>
+        <v>52</v>
       </c>
     </row>
     <row r="23">
@@ -640,7 +643,7 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24">
@@ -650,7 +653,7 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="25">
@@ -660,7 +663,7 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26">
@@ -670,7 +673,7 @@
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="27">
@@ -680,7 +683,7 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="30">
@@ -720,6 +723,16 @@
       </c>
       <c r="B33" s="2" t="n">
         <v>79</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-W30</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -733,7 +746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I198"/>
+  <dimension ref="A1:I229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10053,7 +10066,1465 @@
         </is>
       </c>
     </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t>BrokerTech</t>
+        </is>
+      </c>
+      <c r="C199" s="2" t="inlineStr">
+        <is>
+          <t>Technology &amp; AI</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E199" s="2" t="inlineStr">
+        <is>
+          <t>Vertafore rolls out new AI agents to automate carrier statement reconciliation for agencies</t>
+        </is>
+      </c>
+      <c r="F199" s="2" t="inlineStr">
+        <is>
+          <t>Vertafore released two new Velocity AI agents inside its AgencyOne platform that automate carrier statement reconciliation and turn Outlook email activity into structured workflows, aiming to cut manual work for independent insurance agencies.</t>
+        </is>
+      </c>
+      <c r="G199" s="2" t="inlineStr">
+        <is>
+          <t>PR Newswire</t>
+        </is>
+      </c>
+      <c r="H199" s="2" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/vertafores-latest-ai-innovations-help-agencies-accelerate-carrier-statement-reconciliation-and-turn-outlook-activity-into-structured-workflows-302813535.html</t>
+        </is>
+      </c>
+      <c r="I199" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>BrokerTech</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="inlineStr">
+        <is>
+          <t>People &amp; Leadership</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E200" s="2" t="inlineStr">
+        <is>
+          <t>Fulcrum taps veteran brokerage operations executive to drive AI workflow push</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="inlineStr">
+        <is>
+          <t>Broker-facing AI automation platform Fulcrum brought on a brokerage operations veteran to lead its push into deeper AI workflow adoption, following the company's recent $25 million funding round.</t>
+        </is>
+      </c>
+      <c r="G200" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Business America</t>
+        </is>
+      </c>
+      <c r="H200" s="2" t="inlineStr">
+        <is>
+          <t>https://www.insurancebusinessmag.com/us/news/breaking-news/fulcrum-taps-brokerage-ops-veteran-to-drive-ai-workflow-push-575702.aspx</t>
+        </is>
+      </c>
+      <c r="I200" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B201" s="2" t="inlineStr">
+        <is>
+          <t>Brokers &amp; MGA/GA</t>
+        </is>
+      </c>
+      <c r="C201" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="D201" s="2" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E201" s="2" t="inlineStr">
+        <is>
+          <t>Arrow Global Insurance acquires MGA Fusion Specialty Group</t>
+        </is>
+      </c>
+      <c r="F201" s="2" t="inlineStr">
+        <is>
+          <t>Arrow Global Insurance agreed to acquire managing general agent Fusion Specialty Group, a deal expected to close in the third quarter of 2026 pending regulatory approval, expanding Arrow's specialty program footprint.</t>
+        </is>
+      </c>
+      <c r="G201" s="2" t="inlineStr">
+        <is>
+          <t>The Insurer</t>
+        </is>
+      </c>
+      <c r="H201" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theinsurer.com/program-manager/news/arrow-global-insurance-acquires-mga-fusion-specialty-group-2026-07-09/</t>
+        </is>
+      </c>
+      <c r="I201" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>Brokers &amp; MGA/GA</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>Investments &amp; Funding</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t>American Growth Insurance raises $70 million to acquire and rebuild US brokerages with AI</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t>Tech-forward brokerage growth platform American Growth Insurance raised $70 million in committed equity led by Atomic and Rockbridge Growth Equity, aiming to close several more independent agency acquisitions and rebuild their operations around AI agents.</t>
+        </is>
+      </c>
+      <c r="G202" s="2" t="inlineStr">
+        <is>
+          <t>Beinsure</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="inlineStr">
+        <is>
+          <t>https://beinsure.com/news/american-growth-insurance-raised-70mn/</t>
+        </is>
+      </c>
+      <c r="I202" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B203" s="2" t="inlineStr">
+        <is>
+          <t>Brokers &amp; MGA/GA</t>
+        </is>
+      </c>
+      <c r="C203" s="2" t="inlineStr">
+        <is>
+          <t>People &amp; Leadership</t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t>UK/Europe</t>
+        </is>
+      </c>
+      <c r="E203" s="2" t="inlineStr">
+        <is>
+          <t>PIB Group names Alastair Hay as chief financial officer</t>
+        </is>
+      </c>
+      <c r="F203" s="2" t="inlineStr">
+        <is>
+          <t>UK-based insurance intermediary PIB Group appointed Alastair Hay as its new chief financial officer effective immediately, part of a wave of senior leadership moves across European brokers and MGAs in mid-July.</t>
+        </is>
+      </c>
+      <c r="G203" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Edge</t>
+        </is>
+      </c>
+      <c r="H203" s="2" t="inlineStr">
+        <is>
+          <t>https://insurance-edge.net/2026/07/13/job-moves-and-senior-appointments-13-07-2026/</t>
+        </is>
+      </c>
+      <c r="I203" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>FinTech</t>
+        </is>
+      </c>
+      <c r="C204" s="2" t="inlineStr">
+        <is>
+          <t>Technology &amp; AI</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E204" s="2" t="inlineStr">
+        <is>
+          <t>One Inc and CalcFocus team up to modernize life insurance premium payments</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="inlineStr">
+        <is>
+          <t>Payments network One Inc partnered with policy administration provider CalcFocus to integrate its PremiumPay platform, letting life insurers offer policyholders Apple Pay, Google Pay, PayPal and Venmo alongside traditional card payments.</t>
+        </is>
+      </c>
+      <c r="G204" s="2" t="inlineStr">
+        <is>
+          <t>FinTech Global</t>
+        </is>
+      </c>
+      <c r="H204" s="2" t="inlineStr">
+        <is>
+          <t>https://fintech.global/2026/07/17/one-inc-and-calcfocus-target-friction-in-life-insurance-pay/</t>
+        </is>
+      </c>
+      <c r="I204" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="inlineStr">
+        <is>
+          <t>FinTech</t>
+        </is>
+      </c>
+      <c r="C205" s="2" t="inlineStr">
+        <is>
+          <t>Investments &amp; Funding</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E205" s="2" t="inlineStr">
+        <is>
+          <t>Fulcrum raises $25 million to scale AI automation across US insurance brokers</t>
+        </is>
+      </c>
+      <c r="F205" s="2" t="inlineStr">
+        <is>
+          <t>Fulcrum raised $25 million in seed and Series A funding led by CRV to expand its AI platform for insurance brokers, which automates proposal creation, policy checks and coverage comparisons and has cut policy delivery timelines from 15 days to same-day.</t>
+        </is>
+      </c>
+      <c r="G205" s="2" t="inlineStr">
+        <is>
+          <t>Beinsure</t>
+        </is>
+      </c>
+      <c r="H205" s="2" t="inlineStr">
+        <is>
+          <t>https://beinsure.com/news/fulcrum-raises-25mn-led-by-crv/</t>
+        </is>
+      </c>
+      <c r="I205" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>FinTech</t>
+        </is>
+      </c>
+      <c r="C206" s="2" t="inlineStr">
+        <is>
+          <t>Technology &amp; AI</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E206" s="2" t="inlineStr">
+        <is>
+          <t>PropTech firm Foxen embeds Healthy Paws pet insurance into its renter platform</t>
+        </is>
+      </c>
+      <c r="F206" s="2" t="inlineStr">
+        <is>
+          <t>Foxen partnered with pet insurer Healthy Paws to embed discounted pet coverage directly into its PetClear renter platform, giving qualifying residents a 5% savings on new policies as embedded insurance keeps expanding beyond core financial products.</t>
+        </is>
+      </c>
+      <c r="G206" s="2" t="inlineStr">
+        <is>
+          <t>FinTech Global</t>
+        </is>
+      </c>
+      <c r="H206" s="2" t="inlineStr">
+        <is>
+          <t>https://fintech.global/2026/07/16/foxen-teams-with-healthy-paws-on-renter-pet-insurance/</t>
+        </is>
+      </c>
+      <c r="I206" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t>Health Insurance / Payer</t>
+        </is>
+      </c>
+      <c r="C207" s="2" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E207" s="2" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group's Q2 profit hits $5.4 billion as medical costs ease</t>
+        </is>
+      </c>
+      <c r="F207" s="2" t="inlineStr">
+        <is>
+          <t>UnitedHealth Group reported second-quarter net income of $5.48 billion and raised its 2026 earnings forecast after its medical care ratio fell to 86.7% from 89.4% a year earlier, aided by benefit redesign and exits from unprofitable ACA and Medicare Advantage markets.</t>
+        </is>
+      </c>
+      <c r="G207" s="2" t="inlineStr">
+        <is>
+          <t>Forbes</t>
+        </is>
+      </c>
+      <c r="H207" s="2" t="inlineStr">
+        <is>
+          <t>https://www.forbes.com/sites/brucejapsen/2026/07/16/unitedhealth-group-profits-hit-54-billion-as-costs-continue-to-ease/</t>
+        </is>
+      </c>
+      <c r="I207" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>Health Insurance / Payer</t>
+        </is>
+      </c>
+      <c r="C208" s="2" t="inlineStr">
+        <is>
+          <t>Regulatory &amp; Policy</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E208" s="2" t="inlineStr">
+        <is>
+          <t>FTC secures Caremark settlement locking in up to $8.5 billion in consumer drug savings</t>
+        </is>
+      </c>
+      <c r="F208" s="2" t="inlineStr">
+        <is>
+          <t>The Federal Trade Commission reached a settlement with Caremark Rx and Zinc Health Services resolving claims that the PBM used anticompetitive rebate schemes to inflate insulin prices, requiring rebate pass-through at the point of sale and estimated to save consumers up to $8.5 billion over a decade.</t>
+        </is>
+      </c>
+      <c r="G208" s="2" t="inlineStr">
+        <is>
+          <t>Managed Healthcare Executive</t>
+        </is>
+      </c>
+      <c r="H208" s="2" t="inlineStr">
+        <is>
+          <t>https://www.managedhealthcareexecutive.com/view/ftc-secures-settlement-with-caremark-locks-in-up-to-8-5-billion-in-consumer-savings</t>
+        </is>
+      </c>
+      <c r="I208" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B209" s="2" t="inlineStr">
+        <is>
+          <t>Health Insurance / Payer</t>
+        </is>
+      </c>
+      <c r="C209" s="2" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E209" s="2" t="inlineStr">
+        <is>
+          <t>Health insurers propose median 14% premium increases across ACA exchanges for 2027</t>
+        </is>
+      </c>
+      <c r="F209" s="2" t="inlineStr">
+        <is>
+          <t>Insurers in 16 states and Washington, D.C. have proposed a median 14% premium increase for next year's ACA exchange plans, citing rising healthcare costs and the scheduled expiration of enhanced federal subsidies.</t>
+        </is>
+      </c>
+      <c r="G209" s="2" t="inlineStr">
+        <is>
+          <t>NOTUS</t>
+        </is>
+      </c>
+      <c r="H209" s="2" t="inlineStr">
+        <is>
+          <t>https://www.notus.org/healthcare/health-insurers-are-proposing-to-increase-premiums-again</t>
+        </is>
+      </c>
+      <c r="I209" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t>Healthcare / Provider &amp; Clinical</t>
+        </is>
+      </c>
+      <c r="C210" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E210" s="2" t="inlineStr">
+        <is>
+          <t>Sutter Health and Allina Health sign definitive deal to form $26 billion nonprofit system</t>
+        </is>
+      </c>
+      <c r="F210" s="2" t="inlineStr">
+        <is>
+          <t>Sacramento-based Sutter Health signed a definitive agreement to acquire Minneapolis-based Allina Health, creating a combined 39-hospital, $26 billion nonprofit system spanning California, Minnesota and Wisconsin, with Sutter committing $2 billion to Allina's home markets.</t>
+        </is>
+      </c>
+      <c r="G210" s="2" t="inlineStr">
+        <is>
+          <t>Fierce Healthcare</t>
+        </is>
+      </c>
+      <c r="H210" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fiercehealthcare.com/providers/allina-health-join-sutter-health-26b-proposed-merger</t>
+        </is>
+      </c>
+      <c r="I210" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t>Healthcare / Provider &amp; Clinical</t>
+        </is>
+      </c>
+      <c r="C211" s="2" t="inlineStr">
+        <is>
+          <t>Technology &amp; AI</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E211" s="2" t="inlineStr">
+        <is>
+          <t>Clinical-grade AI moves from data center to point of care as governance infrastructure catches up</t>
+        </is>
+      </c>
+      <c r="F211" s="2" t="inlineStr">
+        <is>
+          <t>A July 2026 digital health roundup finds clinical AI increasingly deployed at the point of care through surgical robots and wearables, with health system leaders emphasizing that strong oversight and clinician accountability determine whether AI strengthens or undermines patient trust.</t>
+        </is>
+      </c>
+      <c r="G211" s="2" t="inlineStr">
+        <is>
+          <t>MarketScale</t>
+        </is>
+      </c>
+      <c r="H211" s="2" t="inlineStr">
+        <is>
+          <t>https://www.marketscale.com/industries/healthcare/digital-healths-july-2026-signal-ai-wearables-a-new-cms-office-and-the-telehealth-billing-fight</t>
+        </is>
+      </c>
+      <c r="I211" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B212" s="2" t="inlineStr">
+        <is>
+          <t>Insurtech</t>
+        </is>
+      </c>
+      <c r="C212" s="2" t="inlineStr">
+        <is>
+          <t>Investments &amp; Funding</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E212" s="2" t="inlineStr">
+        <is>
+          <t>Cover Genius raises $100 million credit facility at $1.9 billion valuation</t>
+        </is>
+      </c>
+      <c r="F212" s="2" t="inlineStr">
+        <is>
+          <t>Embedded insurance platform Cover Genius closed a $100 million credit raise backed by Vista Credit Partners at a $1.9 billion valuation, a sign that embedded insurance financing has matured beyond traditional venture capital rounds.</t>
+        </is>
+      </c>
+      <c r="G212" s="2" t="inlineStr">
+        <is>
+          <t>Tech Times</t>
+        </is>
+      </c>
+      <c r="H212" s="2" t="inlineStr">
+        <is>
+          <t>https://www.techtimes.com/articles/320689/20260716/cover-genius-100m-raise-signals-embedded-insurance-has-outgrown-venture-capital.htm</t>
+        </is>
+      </c>
+      <c r="I212" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t>Insurtech</t>
+        </is>
+      </c>
+      <c r="C213" s="2" t="inlineStr">
+        <is>
+          <t>Technology &amp; AI</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E213" s="2" t="inlineStr">
+        <is>
+          <t>Bamboo Insurance unveils Essential homeowners coverage for straightforward risks</t>
+        </is>
+      </c>
+      <c r="F213" s="2" t="inlineStr">
+        <is>
+          <t>Technology-enabled managing general underwriter Bamboo Insurance launched its Essential homeowners program, an HO2 product built around core coverage for buyers seeking simpler, more affordable protection.</t>
+        </is>
+      </c>
+      <c r="G213" s="2" t="inlineStr">
+        <is>
+          <t>FinTech Global</t>
+        </is>
+      </c>
+      <c r="H213" s="2" t="inlineStr">
+        <is>
+          <t>https://fintech.global/2026/07/06/bamboo-insurance-unveils-essential-homeowners-cover/</t>
+        </is>
+      </c>
+      <c r="I213" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>Investments</t>
+        </is>
+      </c>
+      <c r="C214" s="2" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E214" s="2" t="inlineStr">
+        <is>
+          <t>P&amp;C insurers' book yields hit decade high in 2025 even as income growth cools</t>
+        </is>
+      </c>
+      <c r="F214" s="2" t="inlineStr">
+        <is>
+          <t>Property-casualty insurers' portfolio book yield climbed to a ten-year high of 4.39% in 2025, though net investment income as a share of invested assets slipped modestly from its 2024 peak as reinvestment rates began to normalize.</t>
+        </is>
+      </c>
+      <c r="G214" s="2" t="inlineStr">
+        <is>
+          <t>NEAM</t>
+        </is>
+      </c>
+      <c r="H214" s="2" t="inlineStr">
+        <is>
+          <t>https://www.neamgroup.com/insights/2025-pc-industry-investment-highlights-elevated-yields-persist-as-income-growth-moderates</t>
+        </is>
+      </c>
+      <c r="I214" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
+        <is>
+          <t>Investments</t>
+        </is>
+      </c>
+      <c r="C215" s="2" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E215" s="2" t="inlineStr">
+        <is>
+          <t>Global insurer invested assets climb to $9.6 trillion as insurers keep pivoting toward private markets</t>
+        </is>
+      </c>
+      <c r="F215" s="2" t="inlineStr">
+        <is>
+          <t>A Goldman Sachs Asset Management survey finds US insurers' cash and invested assets grew 6.7% year-over-year to $9.6 trillion at the end of 2025, with respondents expecting continued rotation into private credit and asset-backed finance for incremental yield.</t>
+        </is>
+      </c>
+      <c r="G215" s="2" t="inlineStr">
+        <is>
+          <t>Goldman Sachs Asset Management</t>
+        </is>
+      </c>
+      <c r="H215" s="2" t="inlineStr">
+        <is>
+          <t>https://am.gs.com/en-us/advisors/insights/report-survey/global-insurance-survey</t>
+        </is>
+      </c>
+      <c r="I215" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>Life &amp; Annuities</t>
+        </is>
+      </c>
+      <c r="C216" s="2" t="inlineStr">
+        <is>
+          <t>Regulatory &amp; Policy</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E216" s="2" t="inlineStr">
+        <is>
+          <t>Indexed annuity trade group pushes back on proposed illustration rule changes</t>
+        </is>
+      </c>
+      <c r="F216" s="2" t="inlineStr">
+        <is>
+          <t>The Indexed Annuity Leadership Council submitted comments to the NAIC's Life Insurance and Annuities Illustrations working group opposing parts of a proposed overhaul of Model #245, the annuity disclosure regulation, ahead of further working-group review.</t>
+        </is>
+      </c>
+      <c r="G216" s="2" t="inlineStr">
+        <is>
+          <t>NAIC</t>
+        </is>
+      </c>
+      <c r="H216" s="2" t="inlineStr">
+        <is>
+          <t>https://content.naic.org/sites/default/files/inline-files/ialc-comment.pdf</t>
+        </is>
+      </c>
+      <c r="I216" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t>Life &amp; Annuities</t>
+        </is>
+      </c>
+      <c r="C217" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E217" s="2" t="inlineStr">
+        <is>
+          <t>Life insurers head into second half of 2026 favoring quiet block and reinsurance deals over big mergers</t>
+        </is>
+      </c>
+      <c r="F217" s="2" t="inlineStr">
+        <is>
+          <t>Industry analysts expect life and annuity M&amp;A to stay measured through the rest of 2026, with closed-block transactions, reinsurance arrangements and distribution-driven deals dominating rather than large-scale carrier mergers.</t>
+        </is>
+      </c>
+      <c r="G217" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P Global Market Intelligence</t>
+        </is>
+      </c>
+      <c r="H217" s="2" t="inlineStr">
+        <is>
+          <t>https://www.spglobal.com/market-intelligence/en/news-insights/articles/2026/1/us-life-insurance-2026-outlook-more-closed-block-deals-plenty-of-upside-96755623</t>
+        </is>
+      </c>
+      <c r="I217" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>Property &amp; Casualty</t>
+        </is>
+      </c>
+      <c r="C218" s="2" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E218" s="2" t="inlineStr">
+        <is>
+          <t>Property reinsurance rates fall as much as 25% at July renewals on record capital</t>
+        </is>
+      </c>
+      <c r="F218" s="2" t="inlineStr">
+        <is>
+          <t>Abundant reinsurance capital pushed property catastrophe rates down as much as 25% at the July 1 renewal, with Guy Carpenter's global property rate-on-line index posting its steepest annual decline since the late 1990s.</t>
+        </is>
+      </c>
+      <c r="G218" s="2" t="inlineStr">
+        <is>
+          <t>Business Insurance</t>
+        </is>
+      </c>
+      <c r="H218" s="2" t="inlineStr">
+        <is>
+          <t>https://www.businessinsurance.com/reinsurance-property-renewal-rates-dive-as-much-as-25/</t>
+        </is>
+      </c>
+      <c r="I218" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
+        <is>
+          <t>Property &amp; Casualty</t>
+        </is>
+      </c>
+      <c r="C219" s="2" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E219" s="2" t="inlineStr">
+        <is>
+          <t>US commercial insurance buyers see relief in property and cyber, but casualty costs keep climbing</t>
+        </is>
+      </c>
+      <c r="F219" s="2" t="inlineStr">
+        <is>
+          <t>Alliant's midyear market report finds US commercial buyers getting rate relief in property and cyber lines, while casualty and transportation risks remain pressured by litigation costs and rising claims severity.</t>
+        </is>
+      </c>
+      <c r="G219" s="2" t="inlineStr">
+        <is>
+          <t>The Insurer</t>
+        </is>
+      </c>
+      <c r="H219" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theinsurer.com/ti/news/us-insurance-buyers-see-relief-in-property-cyber-but-casualty-costs-keep-2026-07-20/</t>
+        </is>
+      </c>
+      <c r="I219" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B220" s="2" t="inlineStr">
+        <is>
+          <t>Property &amp; Casualty</t>
+        </is>
+      </c>
+      <c r="C220" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>APAC</t>
+        </is>
+      </c>
+      <c r="E220" s="2" t="inlineStr">
+        <is>
+          <t>KKR joins consortium's A$7.7 billion bid to take Australian broker Steadfast private</t>
+        </is>
+      </c>
+      <c r="F220" s="2" t="inlineStr">
+        <is>
+          <t>KKR joined Amwins Group and Dragoneer Investment Group's non-binding proposal to acquire Australian insurance broker Steadfast Group for roughly A$7.7 billion, with KKR and Dragoneer set to control the retail brokerage business and Amwins taking the underwriting agency operations.</t>
+        </is>
+      </c>
+      <c r="G220" s="2" t="inlineStr">
+        <is>
+          <t>The Insurer</t>
+        </is>
+      </c>
+      <c r="H220" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theinsurer.com/ti/news/kkr-joins-amwins-dragoneer-consortium-bidding-to-acquire-steadfast-2026-07-14/</t>
+        </is>
+      </c>
+      <c r="I220" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B221" s="2" t="inlineStr">
+        <is>
+          <t>Property &amp; Casualty</t>
+        </is>
+      </c>
+      <c r="C221" s="2" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D221" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E221" s="2" t="inlineStr">
+        <is>
+          <t>Excess and surplus lines property rate softening accelerates as casualty increases slow</t>
+        </is>
+      </c>
+      <c r="F221" s="2" t="inlineStr">
+        <is>
+          <t>CRC Group's REDY report shows property rate softening picking up pace in the excess and surplus market even as the rate of casualty rate increases begins to decelerate, reflecting the broader bifurcation in the US commercial market.</t>
+        </is>
+      </c>
+      <c r="G221" s="2" t="inlineStr">
+        <is>
+          <t>The Insurer</t>
+        </is>
+      </c>
+      <c r="H221" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theinsurer.com/e-and-s/news/crc-redy-property-rate-softening-accelerates-as-excess-casualty-increases-slow-2026-07-16/</t>
+        </is>
+      </c>
+      <c r="I221" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B222" s="2" t="inlineStr">
+        <is>
+          <t>Retirement</t>
+        </is>
+      </c>
+      <c r="C222" s="2" t="inlineStr">
+        <is>
+          <t>Regulatory &amp; Policy</t>
+        </is>
+      </c>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E222" s="2" t="inlineStr">
+        <is>
+          <t>India's EPFO formally launches overhauled EPF, pension and insurance schemes for 2026</t>
+        </is>
+      </c>
+      <c r="F222" s="2" t="inlineStr">
+        <is>
+          <t>EPFO rolled out its restructured EPF, EPS and EDLI schemes for 2026 effective July 1, keeping contribution rates unchanged while crediting 8.25% interest on provident fund balances and raising the auto-settlement claims limit to ₹5 lakh.</t>
+        </is>
+      </c>
+      <c r="G222" s="2" t="inlineStr">
+        <is>
+          <t>Business Today</t>
+        </is>
+      </c>
+      <c r="H222" s="2" t="inlineStr">
+        <is>
+          <t>https://www.businesstoday.in/personal-finance/news/story/epfos-new-eps-2026-is-here-whats-changed-for-pensioners-and-epf-subscribers-540351-2026-07-02</t>
+        </is>
+      </c>
+      <c r="I222" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B223" s="2" t="inlineStr">
+        <is>
+          <t>Retirement</t>
+        </is>
+      </c>
+      <c r="C223" s="2" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t>UK/Europe</t>
+        </is>
+      </c>
+      <c r="E223" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;G completes £760 million bulk annuity deal, closing out UK pension scheme's buy-in program</t>
+        </is>
+      </c>
+      <c r="F223" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;G finalized a £760 million bulk purchase annuity with the Smiths Industries Pension Scheme covering more than 10,000 members, the scheme's fifth and final buy-in as UK insurers keep absorbing defined-benefit pension risk.</t>
+        </is>
+      </c>
+      <c r="G223" s="2" t="inlineStr">
+        <is>
+          <t>Insurance Edge</t>
+        </is>
+      </c>
+      <c r="H223" s="2" t="inlineStr">
+        <is>
+          <t>https://insurance-edge.net/2026/07/21/mg-completes-760m-bulk-purchase-annuity-deal/</t>
+        </is>
+      </c>
+      <c r="I223" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B224" s="2" t="inlineStr">
+        <is>
+          <t>Retirement</t>
+        </is>
+      </c>
+      <c r="C224" s="2" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E224" s="2" t="inlineStr">
+        <is>
+          <t>US pension risk transfer deals grow in number but shrink in size as funding surpluses persist</t>
+        </is>
+      </c>
+      <c r="F224" s="2" t="inlineStr">
+        <is>
+          <t>LIMRA data shows the first half of 2026 was marked by a rising count of smaller defined-benefit buy-in transactions even as total US pension risk transfer deal volume edged lower, with insurers still expecting strong appetite for the rest of the year.</t>
+        </is>
+      </c>
+      <c r="G224" s="2" t="inlineStr">
+        <is>
+          <t>Pensions &amp; Investments</t>
+        </is>
+      </c>
+      <c r="H224" s="2" t="inlineStr">
+        <is>
+          <t>https://www.pionline.com/institutional-investors/pension-risk-transfer/pi-limra-pension-risk-transfer-july-2026/</t>
+        </is>
+      </c>
+      <c r="I224" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t>TPA</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E225" s="2" t="inlineStr">
+        <is>
+          <t>Insurance TPA and claims-services businesses fetch 4x-8x EBITDA in 2026 deal market</t>
+        </is>
+      </c>
+      <c r="F225" s="2" t="inlineStr">
+        <is>
+          <t>A new valuation analysis finds founder-led insurance third-party administrator and claims-services firms transacting between 4x and 8x EBITDA in 2026, with revenue type, client concentration and workforce structure driving where deals land in that range.</t>
+        </is>
+      </c>
+      <c r="G225" s="2" t="inlineStr">
+        <is>
+          <t>CT Acquisitions</t>
+        </is>
+      </c>
+      <c r="H225" s="2" t="inlineStr">
+        <is>
+          <t>https://ctacquisitions.com/guides/insurance-tpa-business-valuation/</t>
+        </is>
+      </c>
+      <c r="I225" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
+        <is>
+          <t>Wealth Management</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E226" s="2" t="inlineStr">
+        <is>
+          <t>Wealth Enhancement expands Houston footprint with $299 million Trippon acquisition</t>
+        </is>
+      </c>
+      <c r="F226" s="2" t="inlineStr">
+        <is>
+          <t>Wealth Enhancement closed its purchase of Trippon Wealth Management Group and its affiliated CPA practice, adding roughly $299 million in client assets and pushing the RIA aggregator past $158 billion in total client assets.</t>
+        </is>
+      </c>
+      <c r="G226" s="2" t="inlineStr">
+        <is>
+          <t>InvestmentNews</t>
+        </is>
+      </c>
+      <c r="H226" s="2" t="inlineStr">
+        <is>
+          <t>https://www.investmentnews.com/ria-news/wealth-enhancement-expands-houston-footprint-with-trippon-acquisition/267440</t>
+        </is>
+      </c>
+      <c r="I226" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B227" s="2" t="inlineStr">
+        <is>
+          <t>Wealth Management</t>
+        </is>
+      </c>
+      <c r="C227" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="D227" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E227" s="2" t="inlineStr">
+        <is>
+          <t>Creative Planning bolsters commercial insurance arm with Lovell Insurance Group deal</t>
+        </is>
+      </c>
+      <c r="F227" s="2" t="inlineStr">
+        <is>
+          <t>Creative Planning, a roughly $710 billion RIA, acquired Lee's Summit, Missouri-based commercial insurance brokerage Lovell Insurance Group, continuing a run of specialized acquisitions meant to bring risk-management services to its wealth clients.</t>
+        </is>
+      </c>
+      <c r="G227" s="2" t="inlineStr">
+        <is>
+          <t>InvestmentNews</t>
+        </is>
+      </c>
+      <c r="H227" s="2" t="inlineStr">
+        <is>
+          <t>https://www.investmentnews.com/ria-news/creative-planning-bolsters-commercial-insurance-arm-with-lovell-deal/267443</t>
+        </is>
+      </c>
+      <c r="I227" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B228" s="2" t="inlineStr">
+        <is>
+          <t>Wealth Management</t>
+        </is>
+      </c>
+      <c r="C228" s="2" t="inlineStr">
+        <is>
+          <t>Investments &amp; Funding</t>
+        </is>
+      </c>
+      <c r="D228" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E228" s="2" t="inlineStr">
+        <is>
+          <t>Wealth fintech Arca emerges from stealth with $64 million to build AI-powered advisory platform</t>
+        </is>
+      </c>
+      <c r="F228" s="2" t="inlineStr">
+        <is>
+          <t>Arca, founded by a former Plaid product lead, raised a combined $64 million seed and Series A round led by Venrock and General Catalyst to build AI agents meant to support human financial advisors across planning, tax and estate work.</t>
+        </is>
+      </c>
+      <c r="G228" s="2" t="inlineStr">
+        <is>
+          <t>The AI Insider</t>
+        </is>
+      </c>
+      <c r="H228" s="2" t="inlineStr">
+        <is>
+          <t>https://theaiinsider.tech/2026/07/13/wealth-management-fintech-arca-emerges-from-stealth-with-64-million-to-build-ai-powered-advisory-platform/</t>
+        </is>
+      </c>
+      <c r="I228" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B229" s="2" t="inlineStr">
+        <is>
+          <t>Wealth Management</t>
+        </is>
+      </c>
+      <c r="C229" s="2" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E229" s="2" t="inlineStr">
+        <is>
+          <t>US wealthtech deal count jumps 27% in Q2 2026 even as total funding declines</t>
+        </is>
+      </c>
+      <c r="F229" s="2" t="inlineStr">
+        <is>
+          <t>US wealthtech recorded 116 deals in the second quarter of 2026, up 27% year-over-year, even though total funding fell 41% to $557.8 million as investors favored more, smaller rounds over mega-deals.</t>
+        </is>
+      </c>
+      <c r="G229" s="2" t="inlineStr">
+        <is>
+          <t>FinTech Global</t>
+        </is>
+      </c>
+      <c r="H229" s="2" t="inlineStr">
+        <is>
+          <t>https://fintech.global/2026/07/16/california-emerged-as-the-main-us-wealthtech-hub-in-q2-as-deal-activity-grew-by-27-yoy/</t>
+        </is>
+      </c>
+      <c r="I229" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:I229"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Rebuild rolling 30-day xlsx export with Summary pivot tab
Raw Rows tab has all 889 stories from the last 30 days; Summary tab has
counts by vertical, lens, and ISO week. Counts are written as static
values (computed in Python, equivalent to COUNTIF over the Raw Rows
range) rather than live formulas: this sandbox's LibreOffice hangs
indefinitely in the recalc.py macro step for this workbook, reproduced
even on a minimal styled test file, so shipping formulas would leave
them uncalculated until a human opens the file.
</commit_message>
<xml_diff>
--- a/cockpit-data/story-log-last30days.xlsx
+++ b/cockpit-data/story-log-last30days.xlsx
@@ -46798,9 +46798,8 @@
           <t>Health Insurance / Payer</t>
         </is>
       </c>
-      <c r="B3" s="6">
-        <f>COUNTIF('Raw Rows'!B2:B890,A3)</f>
-        <v/>
+      <c r="B3" s="6" t="n">
+        <v>102</v>
       </c>
     </row>
     <row r="4">
@@ -46809,9 +46808,8 @@
           <t>Healthcare / Provider &amp; Clinical</t>
         </is>
       </c>
-      <c r="B4" s="6">
-        <f>COUNTIF('Raw Rows'!B2:B890,A4)</f>
-        <v/>
+      <c r="B4" s="6" t="n">
+        <v>101</v>
       </c>
     </row>
     <row r="5">
@@ -46820,9 +46818,8 @@
           <t>Property &amp; Casualty</t>
         </is>
       </c>
-      <c r="B5" s="6">
-        <f>COUNTIF('Raw Rows'!B2:B890,A5)</f>
-        <v/>
+      <c r="B5" s="6" t="n">
+        <v>91</v>
       </c>
     </row>
     <row r="6">
@@ -46831,9 +46828,8 @@
           <t>Wealth Management</t>
         </is>
       </c>
-      <c r="B6" s="6">
-        <f>COUNTIF('Raw Rows'!B2:B890,A6)</f>
-        <v/>
+      <c r="B6" s="6" t="n">
+        <v>86</v>
       </c>
     </row>
     <row r="7">
@@ -46842,9 +46838,8 @@
           <t>Brokers &amp; MGA/GA</t>
         </is>
       </c>
-      <c r="B7" s="6">
-        <f>COUNTIF('Raw Rows'!B2:B890,A7)</f>
-        <v/>
+      <c r="B7" s="6" t="n">
+        <v>83</v>
       </c>
     </row>
     <row r="8">
@@ -46853,9 +46848,8 @@
           <t>Life &amp; Annuities</t>
         </is>
       </c>
-      <c r="B8" s="6">
-        <f>COUNTIF('Raw Rows'!B2:B890,A8)</f>
-        <v/>
+      <c r="B8" s="6" t="n">
+        <v>82</v>
       </c>
     </row>
     <row r="9">
@@ -46864,9 +46858,8 @@
           <t>Insurtech</t>
         </is>
       </c>
-      <c r="B9" s="6">
-        <f>COUNTIF('Raw Rows'!B2:B890,A9)</f>
-        <v/>
+      <c r="B9" s="6" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="10">
@@ -46875,9 +46868,8 @@
           <t>Investments</t>
         </is>
       </c>
-      <c r="B10" s="6">
-        <f>COUNTIF('Raw Rows'!B2:B890,A10)</f>
-        <v/>
+      <c r="B10" s="6" t="n">
+        <v>68</v>
       </c>
     </row>
     <row r="11">
@@ -46886,9 +46878,8 @@
           <t>Retirement</t>
         </is>
       </c>
-      <c r="B11" s="6">
-        <f>COUNTIF('Raw Rows'!B2:B890,A11)</f>
-        <v/>
+      <c r="B11" s="6" t="n">
+        <v>61</v>
       </c>
     </row>
     <row r="12">
@@ -46897,9 +46888,8 @@
           <t>BrokerTech</t>
         </is>
       </c>
-      <c r="B12" s="6">
-        <f>COUNTIF('Raw Rows'!B2:B890,A12)</f>
-        <v/>
+      <c r="B12" s="6" t="n">
+        <v>55</v>
       </c>
     </row>
     <row r="13">
@@ -46908,9 +46898,8 @@
           <t>FinTech</t>
         </is>
       </c>
-      <c r="B13" s="6">
-        <f>COUNTIF('Raw Rows'!B2:B890,A13)</f>
-        <v/>
+      <c r="B13" s="6" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="14">
@@ -46919,9 +46908,8 @@
           <t>TPA</t>
         </is>
       </c>
-      <c r="B14" s="6">
-        <f>COUNTIF('Raw Rows'!B2:B890,A14)</f>
-        <v/>
+      <c r="B14" s="6" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="16">
@@ -46949,9 +46937,8 @@
           <t>Market Economics</t>
         </is>
       </c>
-      <c r="B18" s="6">
-        <f>COUNTIF('Raw Rows'!C2:C890,A18)</f>
-        <v/>
+      <c r="B18" s="6" t="n">
+        <v>231</v>
       </c>
     </row>
     <row r="19">
@@ -46960,9 +46947,8 @@
           <t>M&amp;A</t>
         </is>
       </c>
-      <c r="B19" s="6">
-        <f>COUNTIF('Raw Rows'!C2:C890,A19)</f>
-        <v/>
+      <c r="B19" s="6" t="n">
+        <v>151</v>
       </c>
     </row>
     <row r="20">
@@ -46971,9 +46957,8 @@
           <t>Technology &amp; AI</t>
         </is>
       </c>
-      <c r="B20" s="6">
-        <f>COUNTIF('Raw Rows'!C2:C890,A20)</f>
-        <v/>
+      <c r="B20" s="6" t="n">
+        <v>151</v>
       </c>
     </row>
     <row r="21">
@@ -46982,9 +46967,8 @@
           <t>Regulatory &amp; Policy</t>
         </is>
       </c>
-      <c r="B21" s="6">
-        <f>COUNTIF('Raw Rows'!C2:C890,A21)</f>
-        <v/>
+      <c r="B21" s="6" t="n">
+        <v>143</v>
       </c>
     </row>
     <row r="22">
@@ -46993,9 +46977,8 @@
           <t>Investments &amp; Funding</t>
         </is>
       </c>
-      <c r="B22" s="6">
-        <f>COUNTIF('Raw Rows'!C2:C890,A22)</f>
-        <v/>
+      <c r="B22" s="6" t="n">
+        <v>108</v>
       </c>
     </row>
     <row r="23">
@@ -47004,9 +46987,8 @@
           <t>People &amp; Leadership</t>
         </is>
       </c>
-      <c r="B23" s="6">
-        <f>COUNTIF('Raw Rows'!C2:C890,A23)</f>
-        <v/>
+      <c r="B23" s="6" t="n">
+        <v>105</v>
       </c>
     </row>
     <row r="25">
@@ -47034,9 +47016,8 @@
           <t>2026-W27</t>
         </is>
       </c>
-      <c r="B27" s="6">
-        <f>COUNTIF('Raw Rows'!J2:J890,A27)</f>
-        <v/>
+      <c r="B27" s="6" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="28">
@@ -47045,9 +47026,8 @@
           <t>2026-W28</t>
         </is>
       </c>
-      <c r="B28" s="6">
-        <f>COUNTIF('Raw Rows'!J2:J890,A28)</f>
-        <v/>
+      <c r="B28" s="6" t="n">
+        <v>275</v>
       </c>
     </row>
     <row r="29">
@@ -47056,9 +47036,8 @@
           <t>2026-W29</t>
         </is>
       </c>
-      <c r="B29" s="6">
-        <f>COUNTIF('Raw Rows'!J2:J890,A29)</f>
-        <v/>
+      <c r="B29" s="6" t="n">
+        <v>197</v>
       </c>
     </row>
     <row r="30">
@@ -47067,9 +47046,8 @@
           <t>2026-W30</t>
         </is>
       </c>
-      <c r="B30" s="6">
-        <f>COUNTIF('Raw Rows'!J2:J890,A30)</f>
-        <v/>
+      <c r="B30" s="6" t="n">
+        <v>174</v>
       </c>
     </row>
     <row r="31">
@@ -47078,9 +47056,8 @@
           <t>2026-W31</t>
         </is>
       </c>
-      <c r="B31" s="6">
-        <f>COUNTIF('Raw Rows'!J2:J890,A31)</f>
-        <v/>
+      <c r="B31" s="6" t="n">
+        <v>163</v>
       </c>
     </row>
     <row r="32">
@@ -47089,9 +47066,8 @@
           <t>2026-W32</t>
         </is>
       </c>
-      <c r="B32" s="6">
-        <f>COUNTIF('Raw Rows'!J2:J890,A32)</f>
-        <v/>
+      <c r="B32" s="6" t="n">
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily cockpit update 2026-08-14 (Edition #11)
Continues the daily story log from the 2026-08-13 edition (recovered
from branch claude/intelligent-bardeen-cohr9i, the most current
unmerged daily branch) after finding the assigned branch's own history
was five weeks stale.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RoKpSViiYvrMWYiFZY4suV
</commit_message>
<xml_diff>
--- a/cockpit-data/story-log-last30days.xlsx
+++ b/cockpit-data/story-log-last30days.xlsx
@@ -29,20 +29,31 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001A2E40"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="0000294D"/>
       <sz val="16"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="007A8FA3"/>
-      <sz val="9"/>
+      <color rgb="004A5E72"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="004A5E72"/>
-      <sz val="10"/>
+      <color rgb="007A8FA3"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -53,18 +64,8 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <color rgb="001A2E40"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="001A2E40"/>
-      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -80,7 +81,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -88,38 +89,19 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D0D7E0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D0D7E0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D0D7E0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D0D7E0"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -485,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C46"/>
+  <dimension ref="B2:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -503,7 +485,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Window: 2026-07-14 to 2026-08-13  |  Generated: 2026-08-13  |  Rows in window: 27</t>
+          <t>Window: 2026-07-16 to 2026-08-14  |  Generated: 2026-08-14  |  Rows in window: 50</t>
         </is>
       </c>
     </row>
@@ -514,109 +496,99 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="B5" s="4" t="inlineStr">
+    <row r="6">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Counts by Vertical</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" s="5" t="inlineStr">
+    <row r="7">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Vertical</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Stories</t>
         </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>BrokerTech</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Brokers &amp; MGA/GA</t>
+          <t>BrokerTech</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>FinTech</t>
+          <t>Brokers &amp; MGA/GA</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Health Insurance / Payer</t>
+          <t>FinTech</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Healthcare / Provider &amp; Clinical</t>
+          <t>Health Insurance / Payer</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Insurtech</t>
+          <t>Healthcare / Provider &amp; Clinical</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Investments</t>
+          <t>Insurtech</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Life &amp; Annuities</t>
+          <t>Investments</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Property &amp; Casualty</t>
+          <t>Life &amp; Annuities</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
@@ -626,248 +598,258 @@
     <row r="16">
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Retirement</t>
+          <t>Property &amp; Casualty</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>Retirement</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="6" t="inlineStr">
         <is>
+          <t>TPA</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="6" t="inlineStr">
+        <is>
           <t>Wealth Management</t>
         </is>
       </c>
-      <c r="C18" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="4" t="inlineStr">
+      <c r="C19" s="6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="4" t="inlineStr">
+      <c r="C20" s="7" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Counts by Lens</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="5" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>Lens</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Stories</t>
         </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>Investments &amp; Funding</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>M&amp;A</t>
+          <t>Investments &amp; Funding</t>
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Market Economics</t>
+          <t>M&amp;A</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>People &amp; Leadership</t>
+          <t>Market Economics</t>
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Regulatory &amp; Policy</t>
+          <t>People &amp; Leadership</t>
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="6" t="inlineStr">
         <is>
+          <t>Regulatory &amp; Policy</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="6" t="inlineStr">
+        <is>
           <t>Technology &amp; AI</t>
         </is>
       </c>
-      <c r="C29" s="6" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="4" t="inlineStr">
+      <c r="C30" s="6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C30" s="4" t="n">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="4" t="inlineStr">
+      <c r="C31" s="7" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>Counts by Geography</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="5" t="inlineStr">
+    <row r="35">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>Geography</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>Stories</t>
         </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="6" t="inlineStr">
-        <is>
-          <t>APAC</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>APAC</t>
         </is>
       </c>
       <c r="C36" s="6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>UK/Europe</t>
+          <t>India</t>
         </is>
       </c>
       <c r="C38" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="6" t="inlineStr">
         <is>
+          <t>UK/Europe</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="6" t="inlineStr">
+        <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="C39" s="6" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="4" t="inlineStr">
+      <c r="C40" s="6" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="7" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C40" s="4" t="n">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="4" t="inlineStr">
+      <c r="C41" s="7" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>Counts by Week (date_added, ISO week)</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" s="5" t="inlineStr">
+    <row r="45">
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>ISO Week</t>
         </is>
       </c>
-      <c r="C44" s="5" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr">
         <is>
           <t>Stories</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="B45" s="6" t="inlineStr">
+    <row r="46">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>2026-W33</t>
         </is>
       </c>
-      <c r="C45" s="6" t="n">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" s="4" t="inlineStr">
+      <c r="C46" s="6" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="7" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C46" s="4" t="n">
-        <v>27</v>
+      <c r="C47" s="7" t="n">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -881,17 +863,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -943,1271 +925,2352 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Life &amp; Annuities</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>M&amp;A</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>APAC</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>Allianz to buy HSBC Life Singapore for roughly $2bn, locks in 15-year bancassurance tie-up</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Allianz agreed to acquire HSBC Life Singapore for about S$2.7 billion and signed a 15-year exclusive distribution partnership with HSBC Singapore, deepening its foothold in one of Asia's wealthiest insurance markets.</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>Allianz</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>https://www.allianz.com/en/mediacenter/news/media-releases/financials/260724-allianz-to-acquire-hsbc-life-singapore-and-enter-a-new-long-term-distribution-partnership-with-hsbc-singapore.html</t>
         </is>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>2026-07-24</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Life &amp; Annuities</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Market Economics</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>LIC's quarterly profit jumps 23% as new-business margins widen sharply</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>State-run insurer LIC reported a 23% year-on-year rise in first-quarter net profit to roughly Rs 13,492 crore, with value of new business surging 61% and margins expanding nearly 750 basis points.</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>APAC News Network</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>https://apacnewsnetwork.com/2026/08/lic-q1-results-net-profit-jumps-23-percent-to-13492-crore/</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>2026-08-08</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Retirement</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>M&amp;A</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>UK/Europe</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>Standard Life to buy Aegon UK for GBP2bn, creating the UK's largest retirement savings business</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Standard Life agreed to acquire Aegon's UK pensions and savings arm in a GBP2 billion deal, forming a combined retirement business serving 16 million customers with roughly GBP480 billion in assets under administration.</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Professional Pensions</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>https://www.professionalpensions.com/news/4528312/standard-life-buys-aegon-uk-2bn</t>
         </is>
       </c>
-      <c r="I4" s="7" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Retirement</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Technology &amp; AI</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>Retirement Clearinghouse pitches centralized system to fix 401(k) rollover fragmentation</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Retirement Clearinghouse proposed a centralized clearinghouse to address fragmentation in the defined-contribution system, aiming to make it easier for savers to consolidate small accounts when they change jobs or roll into an IRA.</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>WealthManagement.com</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>https://www.wealthmanagement.com/rpa-news/rch-proposes-radical-system-intervention-for-401-k-plans</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>2026-08-01</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Retirement</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Regulatory &amp; Policy</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Neal and Wyden introduce bill cracking down on outsized 'mega' retirement accounts</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>House Ways and Means Ranking Member Richard Neal and Senator Ron Wyden introduced legislation aimed at curbing unusually large IRA and retirement-account balances, part of a broader push on retirement-savings fairness.</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Office of Rep. Richard Neal</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>https://neal.house.gov/2026/07/22/neal-wyden-introduce-bill-to-crack-down-on-mega-retirement-accounts/</t>
         </is>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>2026-07-22</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Investments</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Technology &amp; AI</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>Fidelity to add a guaranteed-income option to its target-date fund lineup</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Fidelity plans to launch Freedom Lifetime, a suite of target-date collective investment trusts with a built-in guaranteed-income feature backed by insurers including Nationwide and New York Life, available to plan sponsors in early 2027.</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>Fidelity Investments</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>https://newsroom.fidelity.com/pressreleases/fidelity-investments--to-expand-target-date-lineup-with-launch-of-guaranteed-income-solution/s/afb7c7fe-f18f-4727-8aa5-3750a24cf9e0</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Investments</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Market Economics</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>Guaranteed-income assets embedded in target-date funds top $100 billion</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Assets tied to guaranteed-income features within target-date funds reached about $103 billion, up 25% from year-end 2024, as more insurers and asset managers partner on in-plan lifetime-income products.</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>401(k) Specialist</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>https://401kspecialistmag.com/guaranteed-income-features-in-target-dates-exceed-100b/</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Wealth Management</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>M&amp;A</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>Carlyle and Bain wage bidding war for $160bn RIA Wealth Enhancement</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Private equity firms Carlyle and Bain Capital are reportedly competing to acquire mega-RIA Wealth Enhancement, which manages roughly $160 billion in client assets, in a deal said to be worth about $7 billion including debt.</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>InvestmentNews</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>https://www.investmentnews.com/ria-news/private-equity-bidding-war-targets-160bn-ria-in-7bn-deal/267559</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Property &amp; Casualty</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Regulatory &amp; Policy</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Allstate seeks Illinois homeowners rate hikes up to 10.4% as losses mount</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Allstate filed for new homeowners rate increases of up to 10.4% affecting more than 200,000 Illinois policyholders, citing severe weather and rising repair costs, reigniting debate over state rate-oversight rules.</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>AM Best / BestWire</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>https://news.ambest.com/newscontent.aspx?AltSrc=23&amp;RefNum=271720</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Property &amp; Casualty</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>M&amp;A</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Mapfre to acquire Safety Insurance in $1.54bn deal, expanding New England reach</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Spanish insurer Mapfre agreed to buy Massachusetts-based Safety Insurance Group in an all-cash $1.54 billion deal at a 44% premium, creating the region's largest homeowners and commercial auto insurer.</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>Insurance Journal</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>https://www.insurancejournal.com/news/east/2026/07/24/878870.htm</t>
         </is>
       </c>
-      <c r="I11" s="7" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>2026-07-24</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Property &amp; Casualty</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Investments &amp; Funding</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Global</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>Zurich secures $1bn reinsurance backstop for its data-center portfolio</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Zurich Insurance entered a new quota-share reinsurance arrangement providing up to $1 billion of capacity to support its fast-growing data-center construction and property book, as AI-driven demand for data-center coverage surges.</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Artemis.bm</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>https://www.artemis.bm/news/zurich-secures-1bn-data-centre-quota-share-breaks-out-us-peak-peril-reinsurance-tower/</t>
         </is>
       </c>
-      <c r="I12" s="7" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Property &amp; Casualty</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Market Economics</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Global</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>Catastrophe bond issuance smashes records as wildfire-exposed deals surge</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Cat bond issuance topped $11 billion in the second quarter, the largest quarter on record, with wildfire-exposed issuance for the year climbing past $5 billion as investor appetite for insurance-linked securities keeps growing.</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Insurance Journal</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>https://www.insurancejournal.com/news/international/2026/08/03/880033.htm</t>
         </is>
       </c>
-      <c r="I13" s="7" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Brokers &amp; MGA/GA</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Investments &amp; Funding</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>AI-native brokerage platform AGI launches with $70 million to buy up agencies</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>American Growth Insurance launched an AI-enabled brokerage growth platform backed by nearly $70 million in committed equity from Rockbridge Growth Equity and Atomic, and closed its first agency acquisition in Baltimore.</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>Insurance Journal</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>https://www.insurancejournal.com/news/southeast/2026/07/20/878204.htm</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>TPA</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Regulatory &amp; Policy</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>New federal law widens fee-disclosure duties to TPAs and stop-loss insurers</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>The Consolidated Appropriations Act of 2026 expanded compensation-disclosure obligations beyond pharmacy benefit managers to cover third-party administrators, stop-loss insurers and most other group health plan service providers, with penalties up to $10,000 a day for noncompliance.</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>Groom Law Group</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>https://www.groom.com/resources/drug-pricing-and-plan-contracting-practices-under-scrutiny-pbm-and-tpa-reforms-in-the-consolidated-appropriations-act-2026/</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>2026-02-03</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>TPA</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Market Economics</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Global</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>Global insurance TPA market keeps expanding as AI-driven claims automation spreads</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>The insurance third-party-administrators market is on track to grow from roughly $372 billion to over $560 billion by 2030, with adoption of AI-driven claims automation and demand for scalable TPA platforms cited as key growth drivers.</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>GlobeNewswire / The Business Research Company</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>https://www.globenewswire.com/news-release/2026/04/27/3281499/28124/en/insurance-third-party-administrators-tpas-global-market-report-2026-yoy-revenue-grew-by-32-billion-ai-driven-claims-automation-to-boost-insurance-tpa-growth-through-2030.html</t>
         </is>
       </c>
-      <c r="I16" s="7" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>2026-04-27</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>FinTech</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Investments &amp; Funding</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>Global</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>Weekly fintech funding cools to $673m across 15 deals</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>Fintech investment pulled back sharply in early August, with $673 million raised across 15 deals, down from more than $2 billion the previous week, though insurance-linked and embedded-finance deals stayed active.</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>FinTech Global</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>https://fintech.global/2026/08/07/a-total-of-673m-was-raised-across-15-fintech-deals-this-week/</t>
         </is>
       </c>
-      <c r="I17" s="7" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>FinTech</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Investments &amp; Funding</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>Global</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>Travel-insurance fintech Faye raises $50m Series C to build an AI travel wallet</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>Faye raised a $50 million Series C led by Madrona at an estimated $500 million valuation, and plans to expand its Faye Wallet product so travelers can manage money and get AI-assisted claims support abroad.</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>FinTech Global</t>
         </is>
       </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>https://fintech.global/2026/08/05/faye-raises-50m-to-build-autonomous-travel-care/</t>
         </is>
       </c>
-      <c r="I18" s="7" t="inlineStr">
+      <c r="I18" s="6" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>BrokerTech</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>Technology &amp; AI</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>BrokerTech Ventures sets Chicago convening for late August with growing sponsor lineup</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>BrokerTech Ventures announced BrokerTech Connect: Chicago, running August 31-September 2, bringing together brokers, carriers, investors and insurtech founders for sessions on AI and the next generation of digital-first insurance organizations.</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>PR Newswire</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/brokertech-connect-chicago-set-for-august-31september-2-announces-growing-sponsor-lineup-and-industry-programming-302848488.html</t>
         </is>
       </c>
-      <c r="I19" s="7" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>BrokerTech</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>People &amp; Leadership</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>Jatin Atre named CEO of insurance software provider Insurity</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>Jatin Atre was appointed chief executive officer of Insurity, succeeding Jeff Clarke, after serving as the company's president since the start of 2026.</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>Insurance Business America</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>https://www.insurancebusinessmag.com/us/news/breaking-news/insurance-moves-insurity-crc-benefits-hdi-global-and-epic-580870.aspx</t>
         </is>
       </c>
-      <c r="I20" s="7" t="inlineStr">
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Insurtech</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Investments &amp; Funding</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>Global</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>Global insurtech funding hits $2.44bn in Q2, the strongest quarter since 2022</t>
         </is>
       </c>
-      <c r="F21" s="8" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>Insurtech funding reached $2.44 billion across 95 deals in the second quarter, the highest quarterly total since 2022, with AI-focused companies capturing nearly all of the available capital, according to Gallagher Re.</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>The Insurer</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>https://www.theinsurer.com/ti/news/insurtech-funding-reaches-244-billion-in-q2-2026-gallagher-re-2026-08-06/</t>
         </is>
       </c>
-      <c r="I21" s="7" t="inlineStr">
+      <c r="I21" s="6" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Insurtech</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>Investments &amp; Funding</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>Ahmedabad insurtech InRisk Labs raises $27m Series A</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>InRisk Labs raised $27 million in a Series A round led by Bessemer Venture Partners and Northpoint Capital, after its reinsurance subsidiary EarthRe became the first incorporated reinsurer licensed at GIFT City's International Financial Services Centre.</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>YourStory</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>https://yourstory.com/2026/08/insurtech-startup-inrisk-labs-raises-27-million-in-series-a</t>
         </is>
       </c>
-      <c r="I22" s="7" t="inlineStr">
+      <c r="I22" s="6" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>Insurtech</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>Technology &amp; AI</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>Global</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>Insurity and ITS partner to close the insurance industry's technology execution gap</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>Insurity and Insurance Technology Services announced a partnership aimed at reducing delivery risk on insurance technology rollouts, targeting the gap between purchasing new insurance software and actually getting it into production.</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>FinTech Global</t>
         </is>
       </c>
-      <c r="H23" s="7" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>https://fintech.global/2026/08/12/insurity-and-its-target-the-insurance-industrys-tech-execution-gap/</t>
         </is>
       </c>
-      <c r="I23" s="7" t="inlineStr">
+      <c r="I23" s="6" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Health Insurance / Payer</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>Market Economics</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>Centene swings to $1.1bn Q2 profit, raises 2026 outlook for the second time this year</t>
         </is>
       </c>
-      <c r="F24" s="8" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>Centene posted $53.6 billion in second-quarter revenue, up 10% year over year, and $1.1 billion in profit, beating expectations as higher premium revenue offset elevated medical costs, prompting another guidance increase.</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>Healthcare Dive</t>
         </is>
       </c>
-      <c r="H24" s="7" t="inlineStr">
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>https://www.healthcaredive.com/news/centene-cnc-q2-2026-guidance-hike-aca-medicaid/826286/</t>
         </is>
       </c>
-      <c r="I24" s="7" t="inlineStr">
+      <c r="I24" s="6" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>Health Insurance / Payer</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>Technology &amp; AI</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>UnitedHealth's Q2 profit hits $5.4bn as it pours $1.5bn into AI cost controls</t>
         </is>
       </c>
-      <c r="F25" s="8" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>UnitedHealth Group reported Q2 profit of $5.4 billion and raised its 2026 adjusted EPS guidance, as the insurer works to stabilize margins by shrinking membership, exiting unprofitable contracts and investing $1.5 billion in AI to streamline operations.</t>
         </is>
       </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>Forbes</t>
         </is>
       </c>
-      <c r="H25" s="7" t="inlineStr">
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>https://www.forbes.com/sites/brucejapsen/2026/07/16/unitedhealth-group-profits-hit-54-billion-as-costs-continue-to-ease/</t>
         </is>
       </c>
-      <c r="I25" s="7" t="inlineStr">
+      <c r="I25" s="6" t="inlineStr">
         <is>
           <t>2026-07-16</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>Healthcare / Provider &amp; Clinical</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>Technology &amp; AI</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>Intermountain Health cuts documentation time 27% with Microsoft's Dragon Copilot</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>Intermountain Health clinicians using Dragon Copilot for 10 or more encounters saw a 27% reduction in time spent on notes per appointment, based on Epic data, as the system scaled the ambient-AI tool across its enterprise.</t>
         </is>
       </c>
-      <c r="G26" s="7" t="inlineStr">
+      <c r="G26" s="6" t="inlineStr">
         <is>
           <t>Microsoft Customer Stories</t>
         </is>
       </c>
-      <c r="H26" s="7" t="inlineStr">
+      <c r="H26" s="6" t="inlineStr">
         <is>
           <t>https://www.microsoft.com/en/customers/story/25891-intermountain-health-microsoft-dragon-copilot</t>
         </is>
       </c>
-      <c r="I26" s="7" t="inlineStr">
+      <c r="I26" s="6" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="inlineStr">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>Healthcare / Provider &amp; Clinical</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>Technology &amp; AI</t>
         </is>
       </c>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="E27" s="8" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>UC Irvine Health warns hospitals often don't know where every AI tool lives in their systems</t>
         </is>
       </c>
-      <c r="F27" s="8" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>UC Irvine Health's chief medical informatics and AI officer, Dr. Deepti Pandita, said provider organizations may not always know where every AI tool exists in their operations, underscoring the need for system-wide AI awareness and governance.</t>
         </is>
       </c>
-      <c r="G27" s="7" t="inlineStr">
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>Odgers Berndtson</t>
         </is>
       </c>
-      <c r="H27" s="7" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>https://www.odgers.com/en-us/insights/ai-operational-governance-an-interview-with-chief-medical-informatics-officer-at-uc-irvine-health-dr-deepti-pandita/</t>
         </is>
       </c>
-      <c r="I27" s="7" t="inlineStr">
+      <c r="I27" s="6" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="inlineStr">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Healthcare / Provider &amp; Clinical</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>Regulatory &amp; Policy</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>UK/Europe</t>
         </is>
       </c>
-      <c r="E28" s="8" t="inlineStr">
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>EU opens EUR9m fund for large-scale clinical AI imaging pilots</t>
         </is>
       </c>
-      <c r="F28" s="8" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>The European Commission's Digital Europe Programme opened a call for proposals worth EUR9 million to fund large-scale pilots of cloud-based AI systems for medical imaging, focused on early detection of cancer and cardiovascular disease in hospitals.</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>European Commission - Digital Strategy</t>
         </is>
       </c>
-      <c r="H28" s="7" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>https://digital-strategy.ec.europa.eu/en/funding/large-scale-pilots-ai-and-genai-medical-imaging</t>
         </is>
       </c>
-      <c r="I28" s="7" t="inlineStr">
+      <c r="I28" s="6" t="inlineStr">
         <is>
           <t>2026-04-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Life &amp; Annuities</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Regulatory &amp; Policy</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>NAIC's life and annuities panel convenes at summer national meeting in Columbus</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>The NAIC Life Insurance and Annuities (A) Committee met August 12 during the 2026 Summer National Meeting in Columbus, Ohio, continuing state regulators' coordination on life and annuity policy priorities.</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>NAIC</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>https://content.naic.org/committees/a/life-insurance-annuities-cmte</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Life &amp; Annuities</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>APAC</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>AIA and Manulife post double-digit new-business growth across Asia</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>AIA's China and Hong Kong operations drove group value of new business up double digits, while Manulife's Asia segment grew core earnings 21% and new business value 13%, both citing strength in Hong Kong, Singapore and mainland China.</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>Insurance Business</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>https://www.insurancebusinessmag.com/asia/news/breaking-news/manulifes-asia-business-grows-core-earnings-21-to-us616-million-in-q2-2026-585128.aspx</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Retirement</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>People &amp; Leadership</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>Voya extends 401(k) recordkeeping deal with law firm Baker Botts</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>Voya Financial renewed its role as recordkeeper for international law firm Baker Botts effective August 1, continuing to serve more than 1,800 plan participants and roughly $900 million in retirement assets.</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>PLANADVISER</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>https://www.planadviser.com/advisory-ma-news-8-12-2026/</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Retirement</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>Target-date fund assets climb to $4.8 trillion as collective trusts gain ground</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>Morningstar's latest target-date fund landscape report found TDF assets rose more than 20% year-over-year to $4.8 trillion, with Vanguard holding about 37% of the market as plan sponsors keep shifting toward lower-cost collective investment trusts.</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>Morningstar (via 401(k) Specialist)</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>https://401kspecialistmag.com/4-8-trillion-and-growing-why-traditional-tdfs-are-still-key-to-401k-success/</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Investments</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Investments &amp; Funding</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>Pimco keeps gathering outside assets as parent Allianz deepens its stake</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>Pimco pulled in EUR31.7 billion of third-party net inflows in the second quarter and continued gathering assets into July, Allianz's CFO said, even as the German insurer increases its ownership position in the asset manager.</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>Bloomberg</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>https://www.bloomberg.com/news/articles/2026-08-07/pimco-keeps-pulling-in-money-as-insurer-allianz-boosts-stake</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Investments</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>Artisan Partners reports $183 billion in assets under management</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>Artisan Partners Asset Management disclosed preliminary assets under management of $183.0 billion as of July 31, 2026, giving an early read on mid-year flows for the publicly traded asset manager.</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>SEC filing (Artisan Partners 8-K)</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/0001517302/000151730226000116/apam-20260811.htm</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>Wealth Management</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>Wealth Enhancement adds $592 million Illinois RIA Miramar Capital</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>Wealth Enhancement acquired the investment advisory business of Miramar Capital, a Northbrook, Illinois-based independent RIA led by Bob Kalman and Max Wasserman that manages more than $592 million in client assets.</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>PR Newswire</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/wealth-enhancement-announces-acquisition-of-miramar-capital-an-independent-ria-with-over-592-million-in-client-assets-302842284.html</t>
+        </is>
+      </c>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Wealth Management</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Investments &amp; Funding</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Carlyle takes minority stake in Prime Capital Financial at $1.8 billion valuation</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>Carlyle's Global Credit platform agreed to roughly a $600 million hybrid capital investment in Prime Capital Financial, valuing the RIA at more than $1.8 billion and letting prior backer Abry Partners exit after three years.</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>InvestmentNews</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>https://www.investmentnews.com/ria-news/carlyle-swoops-in-as-new-prime-capital-backer-valuing-firm-at-18-billion/267735</t>
+        </is>
+      </c>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>Wealth Management</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>People &amp; Leadership</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>Family-office wealthtech Asset Vantage names Nicole Eberhardt global CEO</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>Asset Vantage, an AI-led SaaS platform serving more than 400 families across 10 countries, appointed Nicole Eberhardt as global chief executive effective August 1 to lead its next phase of product and international growth.</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>Hubbis</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>https://www.hubbis.com/news/asset-vantage-appoints-nicole-eberhardt-as-global-chief-executive-officer</t>
+        </is>
+      </c>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Property &amp; Casualty</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>Auto insurance rates resume climbing across more than half of US states</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>After easing in 2025, car insurance premiums are rising again in over half the country, with Connecticut drivers facing the steepest year-over-year increase at 15%, driven by higher repair costs and inflation, per Insurify data.</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>Carrier Management</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>https://www.carriermanagement.com/news/2026/08/13/291037.htm</t>
+        </is>
+      </c>
+      <c r="I38" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>Property &amp; Casualty</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Regulatory &amp; Policy</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>Nevada moves to let home insurers exclude wildfire losses from standard policies</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>Nevada will permit homeowners insurers to carve wildfire coverage out of standard policies starting in 2026, part of a broader wave of state-level moves on wildfire exposure management following record catastrophe losses.</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>AmWINS</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>https://www.amwins.com/resources-and-insights/market-insights/article/state-of-the-market-2026-outlook</t>
+        </is>
+      </c>
+      <c r="I39" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>Brokers &amp; MGA/GA</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>UK/Europe</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>Zurich clears final EU antitrust hurdle for GBP8.1 billion Beazley takeover</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>The European Commission approved Zurich Insurance Group's acquisition of Lloyd's insurer Beazley under simplified merger review; the all-cash deal still needs sign-off from UK, Swiss and Lloyd's regulators.</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>Insurance Times</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>https://www.insurancetimes.co.uk/news/european-commission-clears-zurichs-acquisition-of-beazley/1459100.article</t>
+        </is>
+      </c>
+      <c r="I40" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>Brokers &amp; MGA/GA</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Investments &amp; Funding</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>Reinsurance sidecars and ILS capital step in as traditional reinsurers pull back from MGAs</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>Broker Gallagher Re says growing use of third-party capital, reinsurance sidecars and insurance-linked-securities investors is helping managing general agents replace underwriting capacity that major reinsurers have scaled back.</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>https://www.artemis.bm/news/topic/mga/</t>
+        </is>
+      </c>
+      <c r="I41" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>TPA</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>Fiduciary Services Group buys New Jersey retirement-plan TPA RetireWell</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>Fiduciary Services Group, parent of DWC - The 401(k) Experts, acquired Marlton, NJ-based third-party administrator RetireWell Administrators on July 15, its third TPA acquisition of 2026, adding a firm that services more than 425 retirement plans.</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>PR Newswire</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/fiduciary-services-group-acquires-new-jersey-tpa-retirewell-administrators-302826286.html</t>
+        </is>
+      </c>
+      <c r="I42" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>FinTech</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>Investments &amp; Funding</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>Fisent Technologies raises $4.3 million to scale AI automation for regulated finance firms</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>Fisent Technologies closed a $4.3 million venture round led by FINTOP, with FINTOP partner John Philpott joining its board, to expand its agentic AI platform for banking, insurance and wealth management workflows.</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>GlobeNewswire</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t>https://www.globenewswire.com/news-release/2026/08/11/3342803/0/en/fisent-technologies-accelerates-growth-with-4-3-million-venture-round-to-expand-adoption-of-applied-genai-process-automation-for-regulated-enterprises.html</t>
+        </is>
+      </c>
+      <c r="I43" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>FinTech</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>UK/Europe</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>Cover Genius buys German insurtech Friendsurance to expand DACH bancassurance push</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>Embedded-protection platform Cover Genius acquired Berlin-based Friendsurance, combining its embedded insurance technology with Friendsurance's digital bancassurance and regulatory expertise across Germany, Austria and Switzerland.</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>FinTech Global</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>https://fintech.global/2026/08/03/cover-genius-acquires-friendsurance-to-expand-dach-banking/</t>
+        </is>
+      </c>
+      <c r="I44" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>FinTech</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>APAC</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>SoftBank's PayPay to acquire 70% of T&amp;D Financial Life in AI-driven insurance push</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>PayPay agreed to acquire a 70.2% stake in T&amp;D Financial Life for about JPY134.3 billion ($838 million) as part of a broader alliance with T&amp;D Holdings to distribute insurance through its super-app and develop AI-powered products for Japan's aging population.</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>Japan Times</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>https://www.japantimes.co.jp/business/2026/06/04/softbank-paypay-td-life-insurer/</t>
+        </is>
+      </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>BrokerTech</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Technology &amp; AI</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>SUPERAGENT launches 3.0, billed as an AI 'business partner' for insurance agencies</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>SUPERAGENT released version 3.0 on August 11, replacing traditional agency-software navigation with a conversational AI layer that executes calls, campaigns, renewals and training tasks using live agency data.</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / PRWeb</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/technology/ai/articles/superagent-ai-3-0-launches-121700984.html</t>
+        </is>
+      </c>
+      <c r="I46" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>Insurtech</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Investments &amp; Funding</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>UK/Europe</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>French digital insurer Alan raises EUR480 million at EUR5.5 billion valuation</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>Alan closed a EUR480 million ($550 million) Series G round led by Prosus, with Ontario Teachers' Pension Plan participating for a third straight round, as the profitable French insurer targets Canada as a growth market.</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>The Next Web</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
+          <t>https://thenextweb.com/news/alan-480m-prosus-prevention-insurance</t>
+        </is>
+      </c>
+      <c r="I47" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>Insurtech</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>Technology &amp; AI</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>AI shifts from insurtech pitch to embedded infrastructure, VCs say</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>Roughly 71% of applicants to the 2026 Global InsurTech Competition referenced AI or automation, but investors say the technology is increasingly treated as infrastructure embedded in underwriting and claims workflows rather than a standalone selling point.</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>InsurTechNY</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>https://www.insurtechny.com/insurtech-trends-2026-ai-insurance-startups/</t>
+        </is>
+      </c>
+      <c r="I48" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>Health Insurance / Payer</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>Regulatory &amp; Policy</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>CVS's Caremark settles FTC antitrust case over PBM reimbursement practices</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>CVS Health subsidiaries Caremark Rx and Zinc Health Services agreed to an FTC settlement on July 14 requiring changes to reimbursement practices, making Caremark the second major PBM to resolve enforcement action after Express Scripts settled in February.</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>Federal Trade Commission</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>https://www.ftc.gov/news-events/news/press-releases/2026/07/ftc-secures-major-settlement-caremark-resolving-antitrust-case-against-second-drug-middleman</t>
+        </is>
+      </c>
+      <c r="I49" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>Health Insurance / Payer</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>Regulatory &amp; Policy</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>India weighs national claims exchange and benchmarked treatment rates to curb medical inflation</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>India is considering wide-ranging health insurance reforms, including standardized treatment-rate benchmarks and a nationwide claims exchange, as it seeks to improve transparency amid some of Asia's highest medical inflation.</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>Reuters (via Yahoo News)</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>https://sg.news.yahoo.com/india-plans-insurance-reforms-rein-083021180.html</t>
+        </is>
+      </c>
+      <c r="I50" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>Healthcare / Provider &amp; Clinical</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>Hospital M&amp;A activity rebounds sharply in first half of 2026</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>US hospital and health system mergers rebounded to roughly 40 deals in the first half of 2026, including 18 in the second quarter alone, more than double the same period a year earlier, as systems adjust to new federal and state policy pressures.</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>Chief Healthcare Executive</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>https://www.chiefhealthcareexecutive.com/view/more-hospital-mergers-in-first-half-of-2026-and-momentum-may-continue</t>
+        </is>
+      </c>
+      <c r="I51" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily cockpit update 2026-08-30 (Edition #11)
Adds 25 deduplicated stories across all 12 verticals, 6 lenses and
5 geographies to the persistent story log and today's HTML cockpit.
Also fast-forwards through the previously unmerged 2026-08-29 edition
(PR #52) so this branch carries continuous history instead of another
disconnected day.
</commit_message>
<xml_diff>
--- a/cockpit-data/story-log-last30days.xlsx
+++ b/cockpit-data/story-log-last30days.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Raw Rows (Last 30 Days)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Raw Rows" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,18 +28,25 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="13"/>
+      <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000294D"/>
+        <bgColor rgb="0000294D"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -57,7 +64,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,120 +430,230 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Industry Intelligence Cockpit — Last 30 Days Summary</t>
+          <t>Counts by Vertical</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Counts by Lens</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Counts by Week</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Window: 2026-07-31 to 2026-08-29</t>
-        </is>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>vertical</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>lens</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>week</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Property &amp; Casualty</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>16</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Counts by Vertical</t>
-        </is>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Insurtech</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Technology &amp; AI</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Vertical</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Story Count</t>
-        </is>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Brokers &amp; MGA/GA</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Property &amp; Casualty</t>
+          <t>Health Insurance / Payer</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Investments &amp; Funding</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Brokers &amp; MGA/GA</t>
+          <t>Healthcare / Provider &amp; Clinical</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>6</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Regulatory &amp; Policy</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Health Insurance / Payer</t>
+          <t>FinTech</t>
         </is>
       </c>
       <c r="B8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>People &amp; Leadership</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Retirement</t>
+          <t>Wealth Management</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Investments</t>
+          <t>Retirement</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Wealth Management</t>
+          <t>Life &amp; Annuities</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Insurtech</t>
+          <t>Investments</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Healthcare / Provider &amp; Clinical</t>
+          <t>BrokerTech</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -546,149 +663,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Life &amp; Annuities</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>2</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>FinTech</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>BrokerTech</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>TPA</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Counts by Lens</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Lens</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Story Count</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Market Economics</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>M&amp;A</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Investments &amp; Funding</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Technology &amp; AI</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Regulatory &amp; Policy</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>People &amp; Leadership</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Counts by Week</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>ISO Week</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Story Count</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2026-W35</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -702,17 +681,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -2408,6 +2387,1181 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Life &amp; Annuities</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Top MYGA fixed annuity rates push above 7% in late August</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>The best available multi-year guaranteed annuity rate reached 7.20% simple interest (6.40% compound) on select terms as of August 27, with every rate change that week moving up rather than down even as the Federal Reserve holds a wait-and-see stance.</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>MyAnnuityStore</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>https://myannuitystore.com/annuity-rates/fixed-annuity-rates/</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Life &amp; Annuities</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Regulatory &amp; Policy</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>India advances 100% FDI and policyholder-protection overhaul for insurers</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>IRDAI's 2026 reform package simplifies regulations, strengthens policyholder protection and clears the way for 100% foreign ownership of Indian insurers, with two carriers already raising foreign stakes past the prior 74% cap.</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Vajiram &amp; Ravi</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>https://vajiramandravi.com/current-affairs/irdai-insurance-sector-reforms-2026/</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Retirement</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Pooled Employer Plan adoption jumps 45% as recordkeepers make PEPs a priority</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>PLANADVISER reports 10,797 employers have now adopted Pooled Employer Plans for 401(k) or 403(b) coverage, up from 7,454 a year earlier, with most recordkeepers now ranking PEPs a major or moderate strategic priority.</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>PLANADVISER</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>https://www.planadviser.com/recordkeepers-prioritize-peps-to-spur-growth/</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Retirement</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Regulatory &amp; Policy</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Neal and Wyden target mega retirement accounts as auto-IRA push continues</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Reps. Richard Neal and Ron Wyden introduced legislation to curb oversized retirement accounts, even as Neal separately continues pushing his long-running Automatic IRA Act to auto-enroll workers without employer plans into IRAs or 401(k)s.</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Congressman Richard Neal (House.gov)</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>https://neal.house.gov/2026/07/22/neal-wyden-introduce-bill-to-crack-down-on-mega-retirement-accounts/</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Investments</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>WisdomTree posts sixth straight quarter of record AUM at $162.9 billion</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>WisdomTree's assets under management hit a record $162.9 billion in the second quarter, driven by the Atlantic House acquisition, market appreciation and $3.1 billion of net inflows, marking its sixth consecutive record quarter.</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Pulse2.com</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>https://pulse2.com/wisdomtree-aum-reaches-record-162-9-billion-as-net-inflows-total-3-1-billion/</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Wealth Management</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Apollon and Merit extend RIA buying spree with two more acquisitions</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Apollon Wealth Management added a roughly $650 million RIA while Merit Financial Advisors picked up a $470 million advisory firm, the latest moves in an accelerating wave of RIA consolidation.</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>WealthManagement.com</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>https://www.wealthmanagement.com/ria-news/deals-moves-apollon-adds-650m-ria-merit-snags-470m-advisory</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Wealth Management</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Technology &amp; AI</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>MissionSquare pushes beyond retirement plans into personal wealth management</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>MissionSquare, long focused on public-sector retirement plans, launched a personal wealth management business and rebranded its broker-dealer subsidiary as MissionSquare Wealth Management, naming Shannon Hogendorn as president.</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>FinTech Global</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>https://fintech.global/2026/08/11/missionsquare-expands-into-personal-wealth-management/</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Property &amp; Casualty</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>State Farm raises Illinois home insurance rates 27% on rising claims costs</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>State Farm is raising home insurance rates by an average of 27% for Illinois customers, saying it paid out $1.26 in total costs for every $1 collected in premium in 2024, even as the insurer separately lowers Illinois auto rates.</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>CBS News Chicago</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>https://www.cbsnews.com/chicago/news/state-farm-illinois-home-insurance-rate-hike-august</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Property &amp; Casualty</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>People &amp; Leadership</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>GEICO names Nancy Pierce CEO as insurance leadership shuffle continues</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>GEICO appointed Nancy L. Pierce as chief executive, one of several August leadership changes across the industry that also saw Boston Mutual Life name Grant David Ward CEO and Conduit Holdings name Mark Pickering as incoming CFO.</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Insurance Edge</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>https://insurance-edge.net/2026/08/24/job-moves-and-senior-appointments-24-08-2026/</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Brokers &amp; MGA/GA</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Top five MGA groups now control nearly a fifth of a $17 billion global market</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Brown &amp; Brown, Truist Insurance Holdings, Amwins, Ryan Specialty and Gallagher lead the global MGA, MGU and cover-holder market, which grew roughly 19% to about $17.3 billion in revenue, with Brown &amp; Brown alone topping $1 billion in delegated-underwriting revenue.</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>beinsure.com</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>https://beinsure.com/top-ranking-mga-worldwide/</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Brokers &amp; MGA/GA</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Willis Re agrees to buy BMS Re's US reinsurance division</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Willis Re signed a definitive agreement to acquire the US reinsurance broking and capital-advisory division of BMS Group, calling it a transformational step in accelerating its US expansion.</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Insurance Journal</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>https://www.insurancejournal.com/news/national/2026/08/19/882135.htm</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>TPA</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Technology &amp; AI</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>TPAs push beyond claims handling into prevention and AI-powered risk management</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Gallagher Bassett argues third-party administrators are shifting from reactive claims processing toward proactive risk prevention, pre-loss consulting and AI-driven claims tools as carriers face rising claim severity and complexity.</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Gallagher Bassett</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>https://insurers.gallagherbassett.com/media/beyond-claims-tpas-push-into-prevention-protection-and-ai-powered-risk-management/</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>FinTech</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Technology &amp; AI</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>UK/Europe</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Sixfold partners with Sollers Consulting to speed up AI-driven underwriting</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>AI underwriting insurtech Sixfold teamed up with Sollers Consulting to help carriers combine Sixfold's risk-assessment models with Sollers' implementation expertise for faster underwriting transformation.</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>FinTech Global</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>https://fintech.global/2026/08/14/sixfold-and-sollers-team-up-on-ai-underwriting/</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>FinTech</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Regulatory &amp; Policy</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>UK/Europe</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>EU AI Act's high-risk obligations for insurance underwriting take full effect</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>August 2 marked the date the EU AI Act's high-risk obligations became fully enforceable for uses including credit scoring, insurance underwriting, anti-money-laundering and fraud detection, pushing AI governance to the center of insurers' 2026 strategy.</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>FinTech Global</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>https://fintech.global/2026/08/04/why-ai-governance-is-shaping-insurances-next-phase/</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>FinTech</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Technology &amp; AI</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Insurity and ITS team up to close insurers' technology execution gap</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Insurity partnered with ITS to help carriers move past AI experimentation, targeting the persistent gap between insurers' technology ambitions and their ability to actually execute and scale new systems.</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>FinTech Global</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>https://fintech.global/2026/08/12/insurity-and-its-target-the-insurance-industrys-tech-execution-gap/</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>BrokerTech</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Investments &amp; Funding</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>American Growth Insurance launches AI-enabled brokerage growth platform with $70 million backing</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>American Growth Insurance launched an AI-enabled insurance brokerage growth platform with nearly $70 million in committed equity funding from Rockbridge Growth Equity and venture studio Atomic.</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>PR Newswire</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/american-growth-insurance-launches-specialty-insurance-brokerage-growth-platform-302827676.html</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Insurtech</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Technology &amp; AI</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Bolt debuts what it calls the industry's first AI-powered insurance distribution platform</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Bolt launched Connected Distribution, an AI-driven operating model meant to unify customer data, workflows and market access across all lines of business for its distribution partners.</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>FinTech Global</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>https://fintech.global/2026/08/19/bolt-debuts-industry-first-ai-insurance-platform/</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Insurtech</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Technology &amp; AI</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Carpe launches Minerva Reasoning Engine to help small commercial insurers underwrite profitably</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>AI-native data specialist Carpe introduced its Minerva Reasoning Engine, an underwriting tool aimed specifically at helping small commercial insurers price risk more profitably.</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>FinTech Global</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>https://fintech.global/2026/08/24/carpe-launches-ai-underwriting-tool-for-insurers/</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Insurtech</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>AI adoption and global shocks combine to push insurance pricing higher</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Insurers are citing both the rising cost of AI adoption and a run of global economic and geopolitical shocks as combined pressures pushing premium pricing upward across several lines.</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>FinTech Global</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>https://fintech.global/2026/08/18/ai-and-global-shocks-put-pressure-on-insurance-pricing/</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Insurtech</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Investments &amp; Funding</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>APAC</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Tokio Marine takes minority stake in Singapore insurtech Igloo</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Tokio Marine invested about $5 million for a 1.65% equity stake in Igloo, a full-stack insurtech operating across eight Southeast Asian markets, extending the Japanese carrier's push deeper into the region's digital insurance space.</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Insurance Business Asia</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>https://www.insurancebusinessmag.com/asia/news/technology/tokio-marine-buys-minority-stake-in-singapore-insurtech-igloo-563467.aspx</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Health Insurance / Payer</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Regulatory &amp; Policy</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>CMS backs off proposed Medicare Advantage payment cut, raising 2027 rates nearly 5%</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>CMS finalized Medicare Advantage payment rates for 2027 well above its initial proposal, delivering private insurers close to a 5% average per-enrollee increase after industry pushback on planned cuts.</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>KFF</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>https://www.kff.org/quick-take/medicare-advantage-insurers-will-see-higher-payments-as-cms-backs-off-a-key-payment-update/</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Health Insurance / Payer</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Market Economics</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Insurer exits keep thinning Medicare Advantage options for enrollees</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Becker's Payer Issues tracks a continuing pattern of Medicare Advantage insurer exits and pullbacks in 2026, with a JAMA study finding roughly 10% of MA enrollees had to disenroll and find new coverage after their plans left the market.</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Becker's Payer Issues</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>https://www.beckerspayer.com/payer/medicare-advantage/5-insurers-stepping-back-from-medicare-advantage/</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Healthcare / Provider &amp; Clinical</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Technology &amp; AI</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Innovaccer and AWS strike multi-year deal to scale agentic AI across health systems</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Innovaccer and Amazon Web Services signed a multi-year strategic collaboration aimed at helping health systems and payers move agentic AI from pilot projects into deployments that meet security, compliance and scale requirements.</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Fierce Healthcare</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>https://www.fiercehealthcare.com/health-tech/weekly-rundown-innovaccer-aws-ink-strategic-collab-invoca-launches-patient-engagement</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Healthcare / Provider &amp; Clinical</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Technology &amp; AI</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Exer AI expands Mayo Clinic partnership to widen clinical AI tool deployment</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Exer AI broadened its partnership with Mayo Clinic to further integrate its AI-powered movement-assessment technology into orthopaedic clinical workflows.</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Digital Health News</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>https://www.digitalhealthnews.com/exer-ai-expands-mayo-clinic-partnership-to-advance-clinical-ai-tool-deployment</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Healthcare / Provider &amp; Clinical</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Atrium Health and WakeMed plan combination with $2 billion investment pledge</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Atrium Health, part of Advocate Health, is planning to join forces with WakeMed, pledging $2 billion in investments across Wake County and vowing to create more than 3,000 jobs as large health-system tie-ups continue in 2026.</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Becker's Hospital Review</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>https://www.beckershospitalreview.com/rural-health/growth-merger/11-large-health-systems-growing-bigger/</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>